<commit_message>
Added moduler code for CustomerServiceQA
</commit_message>
<xml_diff>
--- a/Langchain-CustomerServiceQA/data/output.xlsx
+++ b/Langchain-CustomerServiceQA/data/output.xlsx
@@ -516,20 +516,20 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>{'knowledge': {'score': 3, 'reasoning': "The agent's response indicates they are willing to check the issue regarding the double charge, which shows a willingness to assist. However, there is no specific information provided about the customer's concern or any immediate resolution steps. The agent's knowledge about the product or policy is not demonstrated in this interaction, as they did not provide any relevant information or context regarding the charges. Therefore, while the agent is engaging, the lack of detailed knowledge and immediate resolution impacts the overall score."}, 'resolution': {'score': 2, 'reasoning': 'The issue was not fully resolved in the transcript provided. The agent initiated the process of checking the charge but did not confirm whether the double charge was corrected or provide a solution. Follow-up is likely needed to ensure the customer receives a resolution.'}}</t>
+          <t>{'knowledge': {'score': 3, 'reasoning': "The agent's response to the customer's issue of being charged twice is appropriate as they indicate they will check the situation. However, there is no specific information provided regarding the customer's account or the policy in question, which limits the accuracy of the knowledge demonstrated. The agent did not provide any immediate solutions or explanations, which could have improved the interaction."}, 'resolution': {'score': 2, 'reasoning': "The agent acknowledged the issue by checking the customer's account, but there is no indication that the issue was resolved or that a solution was provided. The customer may still be left without clarity on the double charge, and follow-up is likely needed to ensure the issue is addressed."}}</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>The evaluation reveals that the agent demonstrated a willingness to assist the customer with the double charge issue but lacked specific knowledge and immediate resolution steps. The agent's engagement was positive, yet the absence of detailed information and a confirmed resolution negatively impacted the overall effectiveness of the interaction.</t>
+          <t>The evaluation of the agent's performance indicates that while they acknowledged the customer's issue regarding a double charge, their response lacked specific information and immediate solutions. This resulted in a moderate knowledge score and a low resolution score, suggesting that the customer may still be uncertain about the situation.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Enhance training on product knowledge and company policies to ensure agents can provide accurate information regarding charges.
-Implement a checklist for agents to follow during customer interactions to ensure all relevant information is communicated and resolution steps are clearly outlined.
-Encourage agents to confirm resolution of issues before concluding the interaction, ensuring customers leave with a clear understanding of the outcome.
-Provide agents with access to real-time support or resources that can help them quickly address customer concerns during the call.</t>
+          <t>Provide specific account details and relevant policy information to enhance the accuracy of the response.
+Offer immediate solutions or explanations to address the customer's concerns effectively.
+Ensure follow-up communication to confirm that the issue has been resolved and the customer is satisfied.
+Enhance training on handling billing inquiries to improve knowledge and resolution capabilities.</t>
         </is>
       </c>
     </row>
@@ -569,21 +569,20 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>{'knowledge': {'score': 3, 'reasoning': "The agent acknowledged the customer's concern but did not provide specific information regarding the pending claim. While the response was empathetic, it lacked detailed knowledge about the claims process or any actionable steps for the customer. This indicates a moderate level of product/policy knowledge, but the lack of specific guidance affects the overall effectiveness of the response."}, 'resolution': {'score': 2, 'reasoning': "The agent acknowledged the customer's concern but did not provide any specific resolution or information regarding the pending claim. Without a clear solution or next steps, the customer's issue remains unresolved, indicating a low effectiveness in the resolution process."}}</t>
+          <t>{'knowledge': {'score': 3, 'reasoning': "The agent acknowledged the customer's concern but did not provide specific information regarding the pending claim or the reasons for the delay. While the response was empathetic, it lacked detailed product or policy knowledge that could help the customer understand the situation better."}, 'resolution': {'score': 2, 'reasoning': "The agent acknowledged the customer's concern but did not provide a clear resolution or next steps regarding the pending claim. The lack of specific information or a timeline for resolution indicates that the customer's issue remains unresolved, and follow-up is necessary."}}</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>The evaluation of the agent's performance indicates a moderate level of knowledge regarding the claims process, but a significant gap in providing specific information and actionable steps for the customer. The resolution aspect is particularly weak, as the agent failed to offer any clear solutions or next steps, leaving the customer's issue unresolved.</t>
+          <t>The evaluation of the agent's performance indicates a need for improvement in both knowledge and resolution skills. The agent demonstrated empathy but failed to provide specific information about the pending claim, which left the customer without a clear understanding of their situation. Additionally, the agent did not offer a resolution or next steps, resulting in an unresolved issue for the customer.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Enhance training on the claims process to ensure agents can provide specific information and actionable steps.
-Implement role-playing scenarios to practice delivering resolutions effectively and empathetically.
-Encourage agents to ask clarifying questions to better understand customer concerns and provide tailored responses.
-Develop a knowledge base or quick reference guide for agents to access detailed information during customer interactions.
-Monitor and review calls regularly to identify common areas of confusion and provide targeted feedback.</t>
+          <t>Provide training sessions focused on product and policy knowledge to enhance the agent's ability to answer customer inquiries with specific information.
+Implement role-playing scenarios to practice delivering clear resolutions and next steps to customers, ensuring they feel informed and supported.
+Encourage agents to ask clarifying questions to gather necessary details before responding, which can help in providing more accurate and helpful information.
+Establish a follow-up protocol for unresolved issues to ensure that customers receive timely updates on their claims.</t>
         </is>
       </c>
     </row>
@@ -623,21 +622,20 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>{'resolution': {'score': 1, 'reasoning': "The customer's issue remains unresolved after multiple calls, indicating a lack of effective solutions provided by the agent. The agent's apology does not address the specific problem or offer a tangible resolution, suggesting poor service quality. Follow-up is necessary to ensure the customer's issue is addressed."}, 'tone': {'score': 3, 'reasoning': "The agent acknowledges the customer's frustration by apologizing for the inconvenience, which shows some level of empathy. However, the response lacks depth and does not fully address the customer's repeated issues or express a commitment to resolving them, which could enhance the tone of professionalism and emotional appropriateness. The agent's tone is polite but could benefit from more patience and understanding given the customer's escalating frustration."}}</t>
+          <t>{'resolution': {'score': 2, 'reasoning': "The customer's issue remains unresolved after multiple calls, indicating a lack of effective solutions provided by the agent. The agent's apology does not address the root of the problem or offer a concrete resolution, suggesting that follow-up is necessary to ensure the customer's concerns are adequately addressed."}, 'tone': {'score': 4, 'reasoning': "The agent demonstrates professionalism by acknowledging the customer's frustration and apologizing for the inconvenience. This shows a level of empathy towards the customer's situation. However, the response could be improved by providing more specific reassurance or a solution to the issue at hand, which would enhance the perception of patience and emotional appropriateness."}}</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>The evaluation indicates that the customer's issue remains unresolved despite multiple interactions, highlighting a significant gap in the effectiveness of the solutions provided by the agent. While the agent demonstrated some empathy through an apology, the response lacked depth and did not adequately address the customer's ongoing concerns, resulting in a score of 1 for resolution and a score of 3 for tone.</t>
+          <t>The evaluation indicates that the customer's issue remains unresolved despite multiple interactions with the agent. While the agent demonstrates professionalism and empathy, the lack of effective solutions and follow-up is a significant concern. The agent's apology, while appropriate, does not address the core issue or provide a clear path to resolution.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Provide agents with additional training on effective problem-solving techniques to ensure they can offer tangible solutions to customer issues.
-Encourage agents to actively listen to customers and fully understand their concerns before responding, which can help in formulating a more appropriate resolution.
-Implement a follow-up protocol for unresolved issues to ensure that customers feel their concerns are being addressed and to improve overall service quality.
-Enhance training on emotional intelligence to help agents respond with greater empathy and understanding, particularly in situations involving frustrated customers.
-Develop a knowledge base of common issues and effective resolutions that agents can reference during calls to improve their ability to resolve customer problems.</t>
+          <t>Implement training sessions focused on problem-solving techniques to empower agents to provide effective solutions.
+Encourage agents to follow up on unresolved issues to ensure customer concerns are fully addressed.
+Enhance communication skills training to help agents provide specific reassurances and solutions, improving customer satisfaction.
+Develop a checklist for agents to ensure all aspects of a customer's issue are addressed during calls.</t>
         </is>
       </c>
     </row>
@@ -677,20 +675,20 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>{'knowledge': {'score': 4, 'reasoning': "The agent demonstrated a good understanding of the coverage details and was prepared to explain them to the customer. However, without the complete transcript, it's unclear if all the information provided was entirely accurate or if there were any errors in the explanation."}}</t>
+          <t>{'knowledge': {'score': 4, 'reasoning': "The agent demonstrated a good understanding of the coverage details and was prepared to explain them to the customer. However, the transcript does not provide specific details about the coverage, which makes it difficult to fully assess the accuracy of the information provided. Overall, the agent's approach seems knowledgeable, but without specific content, a perfect score cannot be awarded."}}</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>The agent demonstrated a good understanding of coverage details and was able to explain them effectively to the customer. However, the lack of a complete transcript raises concerns about the accuracy of the information provided.</t>
+          <t>The agent demonstrated a good understanding of coverage details and was prepared to explain them to the customer. However, the lack of specific details in the transcript limits the ability to fully assess the accuracy of the information provided. While the agent's approach is knowledgeable, improvements are needed to achieve a perfect score.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Ensure that agents have access to complete transcripts for accurate information delivery.
-Implement regular training sessions focused on coverage details to enhance knowledge retention.
-Encourage agents to verify the accuracy of the information before communicating it to customers.
-Introduce a peer review process for complex customer interactions to ensure accuracy and clarity.</t>
+          <t>Encourage the agent to provide specific details about coverage when discussing with customers to enhance clarity and accuracy.
+Implement training sessions focused on the key aspects of coverage details to ensure agents can confidently relay this information.
+Conduct regular reviews of call transcripts to identify areas where agents can improve their specificity and detail in customer interactions.
+Provide agents with quick reference guides or FAQs that include common coverage details to assist them during customer calls.</t>
         </is>
       </c>
     </row>

</xml_diff>